<commit_message>
Update Splunk Basics - 3 Days Oulines.xlsx
</commit_message>
<xml_diff>
--- a/Splunk Basics - 3 Days Oulines.xlsx
+++ b/Splunk Basics - 3 Days Oulines.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArunKumarHullur\AppData\Local\Microsoft\Windows\INetCache\Content.Outlook\L0JWK38H\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\VK_GIT\SPLK_CISCO_INDIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E725B03C-B136-43EA-8DC9-5D85FF0B76BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{676330DD-14B5-40AD-B417-73DCF815FB93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{A9E713CC-32B9-49A5-A158-F46DA36BDDCD}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A9E713CC-32B9-49A5-A158-F46DA36BDDCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -626,7 +624,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -636,6 +634,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -667,7 +671,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -684,10 +688,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1025,55 +1032,55 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83990E5D-7994-4B9E-BBC0-DA31C75DBE2F}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="59.42578125" customWidth="1"/>
-    <col min="4" max="4" width="50.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="59.44140625" customWidth="1"/>
+    <col min="4" max="4" width="50.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-    </row>
-    <row r="2" spans="1:4" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+    </row>
+    <row r="2" spans="1:4" ht="50.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-    </row>
-    <row r="4" spans="1:4" ht="190.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+    </row>
+    <row r="4" spans="1:4" ht="190.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="5" t="s">
         <v>8</v>
@@ -1085,31 +1092,31 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="165" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="165" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="8" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="165" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="144" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="2" t="s">
         <v>11</v>
@@ -1117,13 +1124,13 @@
       <c r="C8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="8" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="158.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="158.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="8" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -1133,19 +1140,19 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="102.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="102.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>20</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="85.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1153,14 +1160,14 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="135" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="111" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="111" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2" t="s">

</xml_diff>

<commit_message>
user and role document
</commit_message>
<xml_diff>
--- a/Splunk Basics - 3 Days Oulines.xlsx
+++ b/Splunk Basics - 3 Days Oulines.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\VK_GIT\SPLK_CISCO_INDIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFEAB4F8-72AF-4D93-BCE7-37BEC7EB6B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A894910-C993-4ADB-B180-B3D6EAF61402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A9E713CC-32B9-49A5-A158-F46DA36BDDCD}"/>
   </bookViews>
@@ -624,7 +624,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -633,19 +633,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -677,7 +665,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -697,13 +685,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1053,41 +1035,41 @@
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:4" ht="50.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
     </row>
     <row r="4" spans="1:4" ht="190.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
@@ -1103,61 +1085,61 @@
     </row>
     <row r="6" spans="1:4" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="144" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="158.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="102.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="6" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1165,21 +1147,21 @@
       <c r="A11" s="4"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="111" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="6" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>